<commit_message>
V1.03 Minor UI & Template Fixes
</commit_message>
<xml_diff>
--- a/memo/sample_ga_workbook.xlsx
+++ b/memo/sample_ga_workbook.xlsx
@@ -435,29 +435,29 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>Counterparty</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Quarter</t>
-        </is>
-      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>Invoice Link</t>
@@ -475,17 +475,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>UserID</t>
+          <t>USERID</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Descrpn</t>
+          <t>DESCRPN</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>AddlDesc</t>
+          <t>ADDLDESC</t>
         </is>
       </c>
     </row>
@@ -520,29 +520,29 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>Counterparty</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Quarter</t>
-        </is>
-      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>Invoice Link</t>
@@ -560,17 +560,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>UserID</t>
+          <t>USERID</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Descrpn</t>
+          <t>DESCRPN</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>AddlDesc</t>
+          <t>ADDLDESC</t>
         </is>
       </c>
     </row>
@@ -605,29 +605,29 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>Counterparty</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Quarter</t>
-        </is>
-      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>Invoice Link</t>
@@ -645,17 +645,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>UserID</t>
+          <t>USERID</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Descrpn</t>
+          <t>DESCRPN</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>AddlDesc</t>
+          <t>ADDLDESC</t>
         </is>
       </c>
     </row>

</xml_diff>